<commit_message>
ENTG Complete; DCF finished.
</commit_message>
<xml_diff>
--- a/DCFs.xlsx
+++ b/DCFs.xlsx
@@ -2,25 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agnivesh Kaundinya\Desktop\Special Projects\semiconductor-relative-value\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agnivesh Kaundinya\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF16D65-BB47-4AA7-AA48-02FF327754D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D95CDE96-952A-4614-9F48-51E9D579A2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4260" yWindow="390" windowWidth="26610" windowHeight="18345" activeTab="1" xr2:uid="{29E5435A-21FB-4BAD-8CC5-4961AABBFAD0}"/>
+    <workbookView xWindow="4950" yWindow="1080" windowWidth="26610" windowHeight="18345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QCOM" sheetId="1" r:id="rId1"/>
     <sheet name="ENTG" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -32,15 +29,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="79">
   <si>
     <t>QUALCOMM (QCOM) - DCF Model</t>
   </si>
@@ -48,6 +45,9 @@
     <t>All figures $B unless noted</t>
   </si>
   <si>
+    <t>VALUATION DATE: 07/13/2026. MARKET INPUTS FROZEN AS OF THIS DATE.</t>
+  </si>
+  <si>
     <t>Historicals (source: SEC EDGAR 10-Ks)</t>
   </si>
   <si>
@@ -69,6 +69,9 @@
     <t>Capex</t>
   </si>
   <si>
+    <t>NWC</t>
+  </si>
+  <si>
     <t>Assumptions</t>
   </si>
   <si>
@@ -108,6 +111,9 @@
     <t>D%A % of Revenue</t>
   </si>
   <si>
+    <t>NWC % of Revenue</t>
+  </si>
+  <si>
     <t>Selected Case</t>
   </si>
   <si>
@@ -135,24 +141,21 @@
     <t>Less: Capex</t>
   </si>
   <si>
+    <t xml:space="preserve">Less: Change in NWC </t>
+  </si>
+  <si>
     <t>FCF</t>
   </si>
   <si>
-    <t>NWC</t>
-  </si>
-  <si>
-    <t>NWC % of Revenue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Less: Change in NWC </t>
-  </si>
-  <si>
     <t>WACC</t>
   </si>
   <si>
     <t>Risk-Free Rate</t>
   </si>
   <si>
+    <t>Market Risk Premium</t>
+  </si>
+  <si>
     <t>Beta (raw, 5Y monthly)</t>
   </si>
   <si>
@@ -210,6 +213,9 @@
     <t>Plus: Cash</t>
   </si>
   <si>
+    <t>Shares Outstanding (B)</t>
+  </si>
+  <si>
     <t>Intrinsic Value / Share</t>
   </si>
   <si>
@@ -219,12 +225,6 @@
     <t>Upside/(Downside)</t>
   </si>
   <si>
-    <t>Market Risk Premium</t>
-  </si>
-  <si>
-    <t>VALUATION DATE: 07/13/2026. MARKET INPUTS FROZEN AS OF THIS DATE.</t>
-  </si>
-  <si>
     <t>Terminal EBITDA</t>
   </si>
   <si>
@@ -258,18 +258,34 @@
     <t>Implied Terminal Growth</t>
   </si>
   <si>
-    <t>Shares Outstanding (B)</t>
+    <t>ENTEGRIS (ENTG) - DCF Model</t>
+  </si>
+  <si>
+    <t>Operating Margin (Y1)</t>
+  </si>
+  <si>
+    <t>Margin expansion / yr</t>
+  </si>
+  <si>
+    <t>Capex % of Revenue (Y1)</t>
+  </si>
+  <si>
+    <t>Capex change / yr</t>
+  </si>
+  <si>
+    <t>ENTG current EV/EBITDA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-??_);_(@_)"/>
+    <numFmt numFmtId="168" formatCode="[$$-409]#,##0.00;[Red]\-[$$-409]#,##0.00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -277,14 +293,7 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -292,7 +301,14 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -305,7 +321,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -320,33 +336,35 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="2" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Comma" xfId="2" builtinId="3"/>
-    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -366,10 +384,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -407,150 +425,52 @@
         <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
                 <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
                 <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
                 <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
                 <a:lumMod val="102000"/>
                 <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
                 <a:lumMod val="100000"/>
                 <a:shade val="100000"/>
               </a:schemeClr>
@@ -558,33 +478,24 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
                 <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
@@ -597,13 +508,7 @@
           <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -613,15 +518,13 @@
         <a:solidFill>
           <a:schemeClr val="phClr">
             <a:tint val="95000"/>
-            <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
               </a:schemeClr>
@@ -629,7 +532,6 @@
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
               </a:schemeClr>
@@ -637,53 +539,28 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="63000"/>
-                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4F2581F-07E8-4A9E-B536-2BF084D7454F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G113"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.28515625" customWidth="1"/>
     <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="7" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -696,19 +573,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
-        <v>60</v>
+    <row r="3" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5">
         <v>2022</v>
@@ -718,17 +595,17 @@
         <v>2023</v>
       </c>
       <c r="E5">
-        <f t="shared" ref="E5:F5" si="0">D5+1</f>
+        <f>D5+1</f>
         <v>2024</v>
       </c>
       <c r="F5">
-        <f t="shared" si="0"/>
+        <f>E5+1</f>
         <v>2025</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6">
         <v>44.2</v>
@@ -745,7 +622,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7">
         <v>15.86</v>
@@ -762,28 +639,28 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" s="2">
         <f>C7/C6</f>
         <v>0.35882352941176465</v>
       </c>
       <c r="D8" s="2">
-        <f t="shared" ref="D8:F8" si="1">D7/D6</f>
+        <f>D7/D6</f>
         <v>0.21747627024008934</v>
       </c>
       <c r="E8" s="2">
-        <f t="shared" si="1"/>
+        <f>E7/E6</f>
         <v>0.25847022587268992</v>
       </c>
       <c r="F8" s="2">
-        <f t="shared" si="1"/>
+        <f>F7/F6</f>
         <v>0.27913279132791324</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C9">
         <v>1.78</v>
@@ -800,7 +677,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C10">
         <v>2.2599999999999998</v>
@@ -817,7 +694,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C11">
         <v>4.9000000000000004</v>
@@ -834,26 +711,26 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E14" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C15" s="3">
         <v>0</v>
@@ -867,7 +744,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C16" s="3">
         <v>0</v>
@@ -881,7 +758,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C17" s="3">
         <v>-0.01</v>
@@ -895,7 +772,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C18" s="3">
         <v>-0.01</v>
@@ -909,7 +786,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C19" s="3">
         <v>-0.01</v>
@@ -923,7 +800,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C20" s="3">
         <v>0.26</v>
@@ -937,191 +814,191 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C21" s="3">
         <v>0.14000000000000001</v>
       </c>
       <c r="D21" s="3">
-        <f t="shared" ref="D21:E22" si="2">C21</f>
+        <f>C21</f>
         <v>0.14000000000000001</v>
       </c>
       <c r="E21" s="3">
-        <f t="shared" si="2"/>
+        <f>D21</f>
         <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>20</v>
-      </c>
-      <c r="C22" s="1">
+        <v>22</v>
+      </c>
+      <c r="C22" s="4">
         <f>3%</f>
         <v>0.03</v>
       </c>
-      <c r="D22" s="1">
-        <f t="shared" si="2"/>
+      <c r="D22" s="4">
+        <f>C22</f>
         <v>0.03</v>
       </c>
-      <c r="E22" s="1">
-        <f t="shared" si="2"/>
+      <c r="E22" s="4">
+        <f>D22</f>
         <v>0.03</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>21</v>
-      </c>
-      <c r="C23" s="6">
+        <v>23</v>
+      </c>
+      <c r="C23" s="5">
         <f>F9/F6</f>
         <v>3.6585365853658541E-2</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="5">
         <f>C23</f>
         <v>3.6585365853658541E-2</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="5">
         <f>C23</f>
         <v>3.6585365853658541E-2</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>33</v>
-      </c>
-      <c r="C24" s="6">
+        <v>24</v>
+      </c>
+      <c r="C24" s="5">
         <f>$F$11/$F$6</f>
         <v>0.1160794941282746</v>
       </c>
-      <c r="D24" s="6">
-        <f t="shared" ref="D24:E24" si="3">$F$11/$F$6</f>
+      <c r="D24" s="5">
+        <f>$F$11/$F$6</f>
         <v>0.1160794941282746</v>
       </c>
-      <c r="E24" s="6">
-        <f t="shared" si="3"/>
+      <c r="E24" s="5">
+        <f>$F$11/$F$6</f>
         <v>0.1160794941282746</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>22</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>12</v>
+        <v>25</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>14</v>
-      </c>
-      <c r="C28" s="1">
-        <f t="shared" ref="C28:C37" si="4">INDEX($C15:$E15, MATCH($C$26, $C$14:$E$14, 0))</f>
+        <v>16</v>
+      </c>
+      <c r="C28" s="4">
+        <f t="shared" ref="C28:C37" si="0">INDEX($C15:$E15, MATCH($C$26, $C$14:$E$14, 0))</f>
         <v>0.02</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
-        <f>A16</f>
+        <f t="shared" ref="A29:A37" si="1">A16</f>
         <v>Rev growth Y2</v>
       </c>
-      <c r="C29" s="1">
-        <f t="shared" si="4"/>
+      <c r="C29" s="4">
+        <f t="shared" si="0"/>
         <v>0.02</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
-        <f t="shared" ref="A30:A35" si="5">A17</f>
+        <f t="shared" si="1"/>
         <v>Rev growth Y3</v>
       </c>
-      <c r="C30" s="1">
-        <f t="shared" si="4"/>
+      <c r="C30" s="4">
+        <f t="shared" si="0"/>
         <v>0.02</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="1"/>
         <v>Rev growth Y4</v>
       </c>
-      <c r="C31" s="1">
-        <f t="shared" si="4"/>
+      <c r="C31" s="4">
+        <f t="shared" si="0"/>
         <v>0.02</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="1"/>
         <v>Rev growth Y5</v>
       </c>
-      <c r="C32" s="1">
-        <f t="shared" si="4"/>
+      <c r="C32" s="4">
+        <f t="shared" si="0"/>
         <v>0.02</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="1"/>
         <v>Operating Margin</v>
       </c>
-      <c r="C33" s="1">
-        <f t="shared" si="4"/>
+      <c r="C33" s="4">
+        <f t="shared" si="0"/>
         <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="1"/>
         <v>Tax Rate</v>
       </c>
-      <c r="C34" s="1">
-        <f t="shared" si="4"/>
+      <c r="C34" s="4">
+        <f t="shared" si="0"/>
         <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="1"/>
         <v>Capex % of Revenue</v>
       </c>
-      <c r="C35" s="1">
-        <f t="shared" si="4"/>
+      <c r="C35" s="4">
+        <f t="shared" si="0"/>
         <v>0.03</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
-        <f>A23</f>
+        <f t="shared" si="1"/>
         <v>D%A % of Revenue</v>
       </c>
-      <c r="C36" s="6">
-        <f t="shared" si="4"/>
+      <c r="C36" s="5">
+        <f t="shared" si="0"/>
         <v>3.6585365853658541E-2</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
-        <f>A24</f>
+        <f t="shared" si="1"/>
         <v>NWC % of Revenue</v>
       </c>
-      <c r="C37" s="6">
-        <f t="shared" si="4"/>
+      <c r="C37" s="5">
+        <f t="shared" si="0"/>
         <v>0.1160794941282746</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C40">
         <v>2026</v>
@@ -1141,32 +1018,32 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>4</v>
-      </c>
-      <c r="C41" s="5">
+        <v>5</v>
+      </c>
+      <c r="C41" s="7">
         <f>F6*(1+C42)</f>
         <v>45.165600000000005</v>
       </c>
-      <c r="D41" s="5">
+      <c r="D41" s="7">
         <f>C41*(1+D42)</f>
         <v>46.068912000000005</v>
       </c>
-      <c r="E41" s="5">
-        <f t="shared" ref="E41:F41" si="6">D41*(1+E42)</f>
+      <c r="E41" s="7">
+        <f>D41*(1+E42)</f>
         <v>46.990290240000007</v>
       </c>
-      <c r="F41" s="5">
-        <f t="shared" si="6"/>
+      <c r="F41" s="7">
+        <f>E41*(1+F42)</f>
         <v>47.93009604480001</v>
       </c>
-      <c r="G41" s="5">
+      <c r="G41" s="7">
         <f>F41*(1+G42)</f>
         <v>48.888697965696011</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C42" s="3">
         <f>$C$28</f>
@@ -1191,126 +1068,126 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>26</v>
-      </c>
-      <c r="C43" s="5">
+        <v>29</v>
+      </c>
+      <c r="C43" s="7">
         <f>C41*$C$33</f>
         <v>12.646368000000002</v>
       </c>
-      <c r="D43" s="5">
-        <f t="shared" ref="D43:G43" si="7">D41*$C$33</f>
+      <c r="D43" s="7">
+        <f>D41*$C$33</f>
         <v>12.899295360000002</v>
       </c>
-      <c r="E43" s="5">
-        <f t="shared" si="7"/>
+      <c r="E43" s="7">
+        <f>E41*$C$33</f>
         <v>13.157281267200004</v>
       </c>
-      <c r="F43" s="5">
-        <f t="shared" si="7"/>
+      <c r="F43" s="7">
+        <f>F41*$C$33</f>
         <v>13.420426892544004</v>
       </c>
-      <c r="G43" s="5">
-        <f t="shared" si="7"/>
+      <c r="G43" s="7">
+        <f>G41*$C$33</f>
         <v>13.688835430394885</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>27</v>
-      </c>
-      <c r="C44" s="5">
+        <v>30</v>
+      </c>
+      <c r="C44" s="7">
         <f>C43*$C$34</f>
         <v>1.7704915200000004</v>
       </c>
-      <c r="D44" s="5">
-        <f t="shared" ref="D44:G44" si="8">D43*$C$34</f>
+      <c r="D44" s="7">
+        <f>D43*$C$34</f>
         <v>1.8059013504000003</v>
       </c>
-      <c r="E44" s="5">
-        <f t="shared" si="8"/>
+      <c r="E44" s="7">
+        <f>E43*$C$34</f>
         <v>1.8420193774080007</v>
       </c>
-      <c r="F44" s="5">
-        <f t="shared" si="8"/>
+      <c r="F44" s="7">
+        <f>F43*$C$34</f>
         <v>1.8788597649561607</v>
       </c>
-      <c r="G44" s="5">
-        <f t="shared" si="8"/>
+      <c r="G44" s="7">
+        <f>G43*$C$34</f>
         <v>1.9164369602552842</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>28</v>
-      </c>
-      <c r="C45" s="5">
+        <v>31</v>
+      </c>
+      <c r="C45" s="7">
         <f>C43-C44</f>
         <v>10.875876480000002</v>
       </c>
-      <c r="D45" s="5">
-        <f t="shared" ref="D45:G45" si="9">D43-D44</f>
+      <c r="D45" s="7">
+        <f>D43-D44</f>
         <v>11.093394009600001</v>
       </c>
-      <c r="E45" s="5">
-        <f t="shared" si="9"/>
+      <c r="E45" s="7">
+        <f>E43-E44</f>
         <v>11.315261889792003</v>
       </c>
-      <c r="F45" s="5">
-        <f t="shared" si="9"/>
+      <c r="F45" s="7">
+        <f>F43-F44</f>
         <v>11.541567127587843</v>
       </c>
-      <c r="G45" s="5">
-        <f t="shared" si="9"/>
+      <c r="G45" s="7">
+        <f>G43-G44</f>
         <v>11.772398470139601</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>29</v>
-      </c>
-      <c r="C46" s="5">
+        <v>32</v>
+      </c>
+      <c r="C46" s="7">
         <f>C41*$C$36</f>
         <v>1.6524000000000003</v>
       </c>
-      <c r="D46" s="5">
-        <f t="shared" ref="D46:G46" si="10">D41*$C$36</f>
+      <c r="D46" s="7">
+        <f>D41*$C$36</f>
         <v>1.6854480000000003</v>
       </c>
-      <c r="E46" s="5">
-        <f t="shared" si="10"/>
+      <c r="E46" s="7">
+        <f>E41*$C$36</f>
         <v>1.7191569600000005</v>
       </c>
-      <c r="F46" s="5">
-        <f t="shared" si="10"/>
+      <c r="F46" s="7">
+        <f>F41*$C$36</f>
         <v>1.7535400992000005</v>
       </c>
-      <c r="G46" s="5">
-        <f t="shared" si="10"/>
+      <c r="G46" s="7">
+        <f>G41*$C$36</f>
         <v>1.7886109011840006</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>30</v>
-      </c>
-      <c r="C47" s="5">
+        <v>33</v>
+      </c>
+      <c r="C47" s="7">
         <f>C41*$C$35</f>
         <v>1.3549680000000002</v>
       </c>
-      <c r="D47" s="5">
-        <f t="shared" ref="D47:G47" si="11">D41*$C$35</f>
+      <c r="D47" s="7">
+        <f>D41*$C$35</f>
         <v>1.3820673600000002</v>
       </c>
-      <c r="E47" s="5">
-        <f t="shared" si="11"/>
+      <c r="E47" s="7">
+        <f>E41*$C$35</f>
         <v>1.4097087072000001</v>
       </c>
-      <c r="F47" s="5">
-        <f t="shared" si="11"/>
+      <c r="F47" s="7">
+        <f>F41*$C$35</f>
         <v>1.4379028813440002</v>
       </c>
-      <c r="G47" s="5">
-        <f t="shared" si="11"/>
+      <c r="G47" s="7">
+        <f>G41*$C$35</f>
         <v>1.4666609389708802</v>
       </c>
     </row>
@@ -1318,78 +1195,78 @@
       <c r="A48" t="s">
         <v>34</v>
       </c>
-      <c r="C48" s="5">
+      <c r="C48" s="7">
         <f>$C$37*(C41-F6)</f>
         <v>0.10280000000000042</v>
       </c>
-      <c r="D48" s="5">
+      <c r="D48" s="7">
         <f>$C$37*(D41-C41)</f>
         <v>0.10485599999999995</v>
       </c>
-      <c r="E48" s="5">
-        <f t="shared" ref="E48:G48" si="12">$C$37*(E41-D41)</f>
+      <c r="E48" s="7">
+        <f>$C$37*(E41-D41)</f>
         <v>0.10695312000000032</v>
       </c>
-      <c r="F48" s="5">
-        <f t="shared" si="12"/>
+      <c r="F48" s="7">
+        <f>$C$37*(F41-E41)</f>
         <v>0.10909218240000026</v>
       </c>
-      <c r="G48" s="5">
-        <f t="shared" si="12"/>
+      <c r="G48" s="7">
+        <f>$C$37*(G41-F41)</f>
         <v>0.11127402604800012</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>31</v>
-      </c>
-      <c r="C49" s="5">
+        <v>35</v>
+      </c>
+      <c r="C49" s="7">
         <f>C45+C46-C47-C48</f>
         <v>11.070508480000003</v>
       </c>
-      <c r="D49" s="5">
-        <f t="shared" ref="D49:G49" si="13">D45+D46-D47-D48</f>
+      <c r="D49" s="7">
+        <f>D45+D46-D47-D48</f>
         <v>11.291918649600001</v>
       </c>
-      <c r="E49" s="5">
-        <f t="shared" si="13"/>
+      <c r="E49" s="7">
+        <f>E45+E46-E47-E48</f>
         <v>11.517757022592004</v>
       </c>
-      <c r="F49" s="5">
-        <f t="shared" si="13"/>
+      <c r="F49" s="7">
+        <f>F45+F46-F47-F48</f>
         <v>11.748112163043844</v>
       </c>
-      <c r="G49" s="5">
-        <f t="shared" si="13"/>
+      <c r="G49" s="7">
+        <f>G45+G46-G47-G48</f>
         <v>11.98307440630472</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>36</v>
-      </c>
-      <c r="B52" s="1">
+        <v>37</v>
+      </c>
+      <c r="B52" s="4">
         <f>0.0455</f>
         <v>4.5499999999999999E-2</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>59</v>
-      </c>
-      <c r="B53" s="1">
+        <v>38</v>
+      </c>
+      <c r="B53" s="4">
         <f>0.05</f>
         <v>0.05</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B54" s="8">
         <v>1.64</v>
@@ -1397,24 +1274,24 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>38</v>
-      </c>
-      <c r="B55" s="1">
+        <v>40</v>
+      </c>
+      <c r="B55" s="4">
         <f>B52+B53*B54</f>
         <v>0.1275</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>39</v>
-      </c>
-      <c r="B56" s="1">
+        <v>41</v>
+      </c>
+      <c r="B56" s="4">
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B57" s="3">
         <f>C34</f>
@@ -1423,16 +1300,16 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>40</v>
-      </c>
-      <c r="B58" s="1">
+        <v>42</v>
+      </c>
+      <c r="B58" s="4">
         <f>B56*(1-B57)</f>
         <v>4.0677999999999999E-2</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B59">
         <f>185.27*1.054</f>
@@ -1441,7 +1318,7 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B60">
         <v>14.81</v>
@@ -1449,7 +1326,7 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B61">
         <f>B59+B60</f>
@@ -1458,92 +1335,92 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>44</v>
-      </c>
-      <c r="B62" s="1">
+        <v>46</v>
+      </c>
+      <c r="B62" s="4">
         <f>B59/B61</f>
         <v>0.92950458334447961</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>45</v>
-      </c>
-      <c r="B63" s="1">
+        <v>47</v>
+      </c>
+      <c r="B63" s="4">
         <f>B60/B61</f>
         <v>7.0495416655520365E-2</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>35</v>
-      </c>
-      <c r="B64" s="1">
+        <v>36</v>
+      </c>
+      <c r="B64" s="4">
         <f>B62*B55+B63*B58</f>
         <v>0.12137944693513442</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>46</v>
-      </c>
-      <c r="B65" s="7">
+        <v>48</v>
+      </c>
+      <c r="B65" s="9">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C68">
         <f>C40</f>
         <v>2026</v>
       </c>
       <c r="D68">
-        <f t="shared" ref="D68:G68" si="14">D40</f>
+        <f>D40</f>
         <v>2027</v>
       </c>
       <c r="E68">
-        <f t="shared" si="14"/>
+        <f>E40</f>
         <v>2028</v>
       </c>
       <c r="F68">
-        <f t="shared" si="14"/>
+        <f>F40</f>
         <v>2029</v>
       </c>
       <c r="G68">
-        <f t="shared" si="14"/>
+        <f>G40</f>
         <v>2030</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>31</v>
-      </c>
-      <c r="C69" s="5">
+        <v>35</v>
+      </c>
+      <c r="C69" s="7">
         <f>C49</f>
         <v>11.070508480000003</v>
       </c>
-      <c r="D69" s="5">
-        <f t="shared" ref="D69:G69" si="15">D49</f>
+      <c r="D69" s="7">
+        <f>D49</f>
         <v>11.291918649600001</v>
       </c>
-      <c r="E69" s="5">
-        <f t="shared" si="15"/>
+      <c r="E69" s="7">
+        <f>E49</f>
         <v>11.517757022592004</v>
       </c>
-      <c r="F69" s="5">
-        <f t="shared" si="15"/>
+      <c r="F69" s="7">
+        <f>F49</f>
         <v>11.748112163043844</v>
       </c>
-      <c r="G69" s="5">
-        <f t="shared" si="15"/>
+      <c r="G69" s="7">
+        <f>G49</f>
         <v>11.98307440630472</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -1563,32 +1440,32 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>48</v>
-      </c>
-      <c r="C71" s="5">
+        <v>50</v>
+      </c>
+      <c r="C71" s="7">
         <f>-PV($B$64, C70, 0, C69)</f>
         <v>9.8722234567942557</v>
       </c>
-      <c r="D71" s="5">
-        <f t="shared" ref="D71:G71" si="16">-PV($B$64, D70, 0, D69)</f>
+      <c r="D71" s="7">
+        <f>-PV($B$64, D70, 0, D69)</f>
         <v>8.9797150763301037</v>
       </c>
-      <c r="E71" s="5">
-        <f t="shared" si="16"/>
+      <c r="E71" s="7">
+        <f>-PV($B$64, E70, 0, E69)</f>
         <v>8.1678948217663603</v>
       </c>
-      <c r="F71" s="5">
-        <f t="shared" si="16"/>
+      <c r="F71" s="7">
+        <f>-PV($B$64, F70, 0, F69)</f>
         <v>7.4294680011944303</v>
       </c>
-      <c r="G71" s="5">
-        <f t="shared" si="16"/>
+      <c r="G71" s="7">
+        <f>-PV($B$64, G70, 0, G69)</f>
         <v>6.7577994067307596</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B73">
         <f>(G69*(1+$B$65))/($B$64-$B$65)</f>
@@ -1597,7 +1474,7 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B74" s="8">
         <f>-PV(B64, 5, 0, B73)</f>
@@ -1606,25 +1483,25 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>51</v>
-      </c>
-      <c r="B75" s="5">
+        <v>53</v>
+      </c>
+      <c r="B75" s="7">
         <f>SUM(C71:G71)</f>
         <v>41.207100762815912</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>52</v>
-      </c>
-      <c r="B76" s="9">
+        <v>54</v>
+      </c>
+      <c r="B76" s="10">
         <f>B74+B75</f>
         <v>113.07661871679302</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B77">
         <f>B74/B76</f>
@@ -1633,16 +1510,16 @@
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>52</v>
-      </c>
-      <c r="B79" s="9">
+        <v>54</v>
+      </c>
+      <c r="B79" s="10">
         <f>B76</f>
         <v>113.07661871679302</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B80">
         <f>B60</f>
@@ -1651,7 +1528,7 @@
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B81">
         <f>5520000000/1000000000+4.63</f>
@@ -1660,16 +1537,16 @@
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>41</v>
-      </c>
-      <c r="B82" s="9">
+        <v>43</v>
+      </c>
+      <c r="B82" s="10">
         <f>B79-B80+B81</f>
         <v>108.41661871679301</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="B83" s="8">
         <f>1054000000/1000000000</f>
@@ -1678,7 +1555,7 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B84">
         <f>(B82)/B83</f>
@@ -1687,7 +1564,7 @@
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B85">
         <v>185.27</v>
@@ -1695,7 +1572,7 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B86">
         <f>B84/B85-1</f>
@@ -1704,18 +1581,18 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C89" s="3">
         <v>0.02</v>
       </c>
-      <c r="D89" s="7">
+      <c r="D89" s="9">
         <v>2.2499999999999999E-2</v>
       </c>
-      <c r="E89" s="7">
+      <c r="E89" s="9">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F89" s="7">
+      <c r="F89" s="9">
         <v>2.75E-2</v>
       </c>
       <c r="G89" s="3">
@@ -1723,198 +1600,198 @@
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B90" s="10">
+      <c r="B90" s="11">
         <v>0.1</v>
       </c>
-      <c r="C90" s="11">
-        <f>(NPV($B90,$C$69:$G$69)+(($G$69*(1+C$89))/($B90-C$89))/(1+$B90)^5-$B$60+$B$81)/$B$83</f>
+      <c r="C90" s="12">
+        <f t="shared" ref="C90:G96" si="2">(NPV($B90,$C$69:$G$69)+(($G$69*(1+C$89))/($B90-C$89))/(1+$B90)^5-$B$60+$B$81)/$B$83</f>
         <v>126.87035673624287</v>
       </c>
-      <c r="D90" s="11">
-        <f t="shared" ref="D90:G96" si="17">(NPV($B90,$C$69:$G$69)+(($G$69*(1+D$89))/($B90-D$89))/(1+$B90)^5-$B$60+$B$81)/$B$83</f>
+      <c r="D90" s="12">
+        <f t="shared" si="2"/>
         <v>130.00151647186863</v>
       </c>
-      <c r="E90" s="11">
-        <f t="shared" si="17"/>
+      <c r="E90" s="12">
+        <f t="shared" si="2"/>
         <v>133.34142018986944</v>
       </c>
-      <c r="F90" s="11">
-        <f t="shared" si="17"/>
+      <c r="F90" s="12">
+        <f t="shared" si="2"/>
         <v>136.91166209531863</v>
       </c>
-      <c r="G90" s="11">
-        <f t="shared" si="17"/>
+      <c r="G90" s="12">
+        <f t="shared" si="2"/>
         <v>140.73692127972845</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B91" s="10">
-        <f>B90+0.5%</f>
+      <c r="B91" s="11">
+        <f t="shared" ref="B91:B96" si="3">B90+0.5%</f>
         <v>0.10500000000000001</v>
       </c>
-      <c r="C91" s="11">
-        <f t="shared" ref="C91:C96" si="18">(NPV($B91,$C$69:$G$69)+(($G$69*(1+C$89))/($B91-C$89))/(1+$B91)^5-$B$60+$B$81)/$B$83</f>
+      <c r="C91" s="12">
+        <f t="shared" si="2"/>
         <v>119.14732090635118</v>
       </c>
-      <c r="D91" s="11">
-        <f t="shared" si="17"/>
+      <c r="D91" s="12">
+        <f t="shared" si="2"/>
         <v>121.86592312775092</v>
       </c>
-      <c r="E91" s="11">
-        <f t="shared" si="17"/>
+      <c r="E91" s="12">
+        <f t="shared" si="2"/>
         <v>124.75443798798815</v>
       </c>
-      <c r="F91" s="11">
-        <f t="shared" si="17"/>
+      <c r="F91" s="12">
+        <f t="shared" si="2"/>
         <v>127.82930864566009</v>
       </c>
-      <c r="G91" s="11">
-        <f t="shared" si="17"/>
+      <c r="G91" s="12">
+        <f t="shared" si="2"/>
         <v>131.10917068051015</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B92" s="10">
-        <f t="shared" ref="B92:B96" si="19">B91+0.5%</f>
+      <c r="B92" s="11">
+        <f t="shared" si="3"/>
         <v>0.11000000000000001</v>
       </c>
-      <c r="C92" s="11">
-        <f t="shared" si="18"/>
+      <c r="C92" s="12">
+        <f t="shared" si="2"/>
         <v>112.2824001686696</v>
       </c>
-      <c r="D92" s="11">
-        <f t="shared" si="17"/>
+      <c r="D92" s="12">
+        <f t="shared" si="2"/>
         <v>114.65992562781753</v>
       </c>
-      <c r="E92" s="11">
-        <f t="shared" si="17"/>
+      <c r="E92" s="12">
+        <f t="shared" si="2"/>
         <v>117.17730552573892</v>
       </c>
-      <c r="F92" s="11">
-        <f t="shared" si="17"/>
+      <c r="F92" s="12">
+        <f t="shared" si="2"/>
         <v>119.84725390232218</v>
       </c>
-      <c r="G92" s="11">
-        <f t="shared" si="17"/>
+      <c r="G92" s="12">
+        <f t="shared" si="2"/>
         <v>122.68407405244189</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B93" s="10">
-        <f t="shared" si="19"/>
+      <c r="B93" s="11">
+        <f t="shared" si="3"/>
         <v>0.11500000000000002</v>
       </c>
-      <c r="C93" s="11">
-        <f t="shared" si="18"/>
+      <c r="C93" s="12">
+        <f t="shared" si="2"/>
         <v>106.14010266653349</v>
       </c>
-      <c r="D93" s="11">
-        <f t="shared" si="17"/>
+      <c r="D93" s="12">
+        <f t="shared" si="2"/>
         <v>108.23278277490434</v>
       </c>
-      <c r="E93" s="11">
-        <f t="shared" si="17"/>
+      <c r="E93" s="12">
+        <f t="shared" si="2"/>
         <v>110.4417228892958</v>
       </c>
-      <c r="F93" s="11">
-        <f t="shared" si="17"/>
+      <c r="F93" s="12">
+        <f t="shared" si="2"/>
         <v>112.77688815308106</v>
       </c>
-      <c r="G93" s="11">
-        <f t="shared" si="17"/>
+      <c r="G93" s="12">
+        <f t="shared" si="2"/>
         <v>115.24941607944191</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B94" s="10">
-        <f t="shared" si="19"/>
+      <c r="B94" s="11">
+        <f t="shared" si="3"/>
         <v>0.12000000000000002</v>
       </c>
-      <c r="C94" s="11">
-        <f t="shared" si="18"/>
+      <c r="C94" s="12">
+        <f t="shared" si="2"/>
         <v>100.61203491461099</v>
       </c>
-      <c r="D94" s="11">
-        <f t="shared" si="17"/>
+      <c r="D94" s="12">
+        <f t="shared" si="2"/>
         <v>102.46467453414995</v>
       </c>
-      <c r="E94" s="12">
-        <f t="shared" si="17"/>
+      <c r="E94" s="13">
+        <f t="shared" si="2"/>
         <v>104.4148215020857</v>
       </c>
-      <c r="F94" s="11">
-        <f t="shared" si="17"/>
+      <c r="F94" s="12">
+        <f t="shared" si="2"/>
         <v>106.47038181963963</v>
       </c>
-      <c r="G94" s="11">
-        <f t="shared" si="17"/>
+      <c r="G94" s="12">
+        <f t="shared" si="2"/>
         <v>108.64013993261317</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B95" s="10">
-        <f>B94+0.5%</f>
+      <c r="B95" s="11">
+        <f t="shared" si="3"/>
         <v>0.12500000000000003</v>
       </c>
-      <c r="C95" s="11">
-        <f t="shared" si="18"/>
+      <c r="C95" s="12">
+        <f t="shared" si="2"/>
         <v>95.610449805728749</v>
       </c>
-      <c r="D95" s="11">
-        <f t="shared" si="17"/>
+      <c r="D95" s="12">
+        <f t="shared" si="2"/>
         <v>97.259160289505147</v>
       </c>
-      <c r="E95" s="11">
-        <f t="shared" si="17"/>
+      <c r="E95" s="12">
+        <f t="shared" si="2"/>
         <v>98.990306297470369</v>
       </c>
-      <c r="F95" s="11">
-        <f t="shared" si="17"/>
+      <c r="F95" s="12">
+        <f t="shared" si="2"/>
         <v>100.8102290237928</v>
       </c>
-      <c r="G95" s="11">
-        <f t="shared" si="17"/>
+      <c r="G95" s="12">
+        <f t="shared" si="2"/>
         <v>102.72593715676376</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B96" s="10">
-        <f t="shared" si="19"/>
+      <c r="B96" s="11">
+        <f t="shared" si="3"/>
         <v>0.13000000000000003</v>
       </c>
-      <c r="C96" s="11">
-        <f t="shared" si="18"/>
+      <c r="C96" s="12">
+        <f t="shared" si="2"/>
         <v>91.063554252199367</v>
       </c>
-      <c r="D96" s="11">
-        <f t="shared" si="17"/>
+      <c r="D96" s="12">
+        <f t="shared" si="2"/>
         <v>92.537741772721617</v>
       </c>
-      <c r="E96" s="11">
-        <f t="shared" si="17"/>
+      <c r="E96" s="12">
+        <f t="shared" si="2"/>
         <v>94.082128698983027</v>
       </c>
-      <c r="F96" s="11">
-        <f t="shared" si="17"/>
+      <c r="F96" s="12">
+        <f t="shared" si="2"/>
         <v>95.701851572866985</v>
       </c>
-      <c r="G96" s="11">
-        <f t="shared" si="17"/>
+      <c r="G96" s="12">
+        <f t="shared" si="2"/>
         <v>97.402560590445106</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>61</v>
-      </c>
-      <c r="B99" s="5">
+        <v>62</v>
+      </c>
+      <c r="B99" s="7">
         <f>G43+G46</f>
         <v>15.477446331578886</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B100">
         <f>B73/B99</f>
@@ -1923,7 +1800,7 @@
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B101">
         <f>(B59+B60-B81)/(F7+F9)</f>
@@ -1932,7 +1809,7 @@
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C104">
         <v>8</v>
@@ -1952,73 +1829,73 @@
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>65</v>
-      </c>
-      <c r="C105">
+        <v>66</v>
+      </c>
+      <c r="C105" s="14">
         <f>(NPV($B$64,$C$69:$G$69)+(C104*$B$99)/(1+$B$64)^5-$B$60+$B$81)/$B$83</f>
         <v>100.9246443478747</v>
       </c>
-      <c r="D105">
-        <f t="shared" ref="D105:G105" si="20">(NPV($B$64,$C$69:$G$69)+(D104*$B$99)/(1+$B$64)^5-$B$60+$B$81)/$B$83</f>
+      <c r="D105" s="14">
+        <f>(NPV($B$64,$C$69:$G$69)+(D104*$B$99)/(1+$B$64)^5-$B$60+$B$81)/$B$83</f>
         <v>117.48713827098761</v>
       </c>
-      <c r="E105">
-        <f t="shared" si="20"/>
+      <c r="E105" s="14">
+        <f>(NPV($B$64,$C$69:$G$69)+(E104*$B$99)/(1+$B$64)^5-$B$60+$B$81)/$B$83</f>
         <v>134.04963219410052</v>
       </c>
-      <c r="F105">
-        <f t="shared" si="20"/>
+      <c r="F105" s="14">
+        <f>(NPV($B$64,$C$69:$G$69)+(F104*$B$99)/(1+$B$64)^5-$B$60+$B$81)/$B$83</f>
         <v>158.89337307876991</v>
       </c>
-      <c r="G105">
-        <f t="shared" si="20"/>
+      <c r="G105" s="14">
+        <f>(NPV($B$64,$C$69:$G$69)+(G104*$B$99)/(1+$B$64)^5-$B$60+$B$81)/$B$83</f>
         <v>183.7371139634393</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>67</v>
-      </c>
-      <c r="B109" s="9">
+        <v>68</v>
+      </c>
+      <c r="B109" s="10">
         <f>B85*B83</f>
         <v>195.27458000000001</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>68</v>
-      </c>
-      <c r="B110" s="9">
+        <v>69</v>
+      </c>
+      <c r="B110" s="10">
         <f>B109+B60-B81</f>
         <v>199.93458000000001</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>69</v>
-      </c>
-      <c r="B111" s="9">
+        <v>70</v>
+      </c>
+      <c r="B111" s="10">
         <f>(B110-B75)*(1+B64)^5</f>
         <v>281.45896016533607</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>70</v>
-      </c>
-      <c r="B112" s="9">
+        <v>71</v>
+      </c>
+      <c r="B112" s="10">
         <f>B111/B99</f>
         <v>18.185103287424798</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B113" s="2">
         <f>(B64*B111-G69*(1+0))/(B111+G69)</f>
@@ -2026,16 +1903,1463 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD674BD-0641-40E2-8223-3020DF8EF03C}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:G119"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="38.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>2022</v>
+      </c>
+      <c r="D5">
+        <f>C5+1</f>
+        <v>2023</v>
+      </c>
+      <c r="E5">
+        <f>D5+1</f>
+        <v>2024</v>
+      </c>
+      <c r="F5">
+        <f>E5+1</f>
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>3.28</v>
+      </c>
+      <c r="D6">
+        <v>3.52</v>
+      </c>
+      <c r="E6">
+        <v>3.24</v>
+      </c>
+      <c r="F6">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>0.48</v>
+      </c>
+      <c r="D7">
+        <v>0.5</v>
+      </c>
+      <c r="E7">
+        <v>0.53</v>
+      </c>
+      <c r="F7">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="9">
+        <f>C7/C6</f>
+        <v>0.14634146341463414</v>
+      </c>
+      <c r="D8" s="9">
+        <f>D7/D6</f>
+        <v>0.14204545454545456</v>
+      </c>
+      <c r="E8" s="9">
+        <f>E7/E6</f>
+        <v>0.16358024691358025</v>
+      </c>
+      <c r="F8" s="9">
+        <f>F7/F6</f>
+        <v>0.14374999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="D9">
+        <v>0.39</v>
+      </c>
+      <c r="E9">
+        <v>0.38</v>
+      </c>
+      <c r="F9">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>0.47</v>
+      </c>
+      <c r="D10">
+        <v>0.46</v>
+      </c>
+      <c r="E10">
+        <v>0.32</v>
+      </c>
+      <c r="F10">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>0.79</v>
+      </c>
+      <c r="E11">
+        <v>0.82</v>
+      </c>
+      <c r="F11">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.06</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0.06</v>
+      </c>
+      <c r="E16" s="3">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="E19" s="3">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="3">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0.17</v>
+      </c>
+      <c r="E20" s="3">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>75</v>
+      </c>
+      <c r="C21" s="9">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="D21" s="9">
+        <v>0.01</v>
+      </c>
+      <c r="E21" s="9">
+        <v>1.2500000000000001E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="3">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="D22" s="3">
+        <f t="shared" ref="D22:E24" si="0">C22</f>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E22" s="3">
+        <f t="shared" si="0"/>
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" s="3">
+        <f>8%</f>
+        <v>0.08</v>
+      </c>
+      <c r="D23" s="3">
+        <f t="shared" si="0"/>
+        <v>0.08</v>
+      </c>
+      <c r="E23" s="3">
+        <f t="shared" si="0"/>
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" s="9">
+        <v>-5.0000000000000001E-3</v>
+      </c>
+      <c r="D24" s="9">
+        <f t="shared" si="0"/>
+        <v>-5.0000000000000001E-3</v>
+      </c>
+      <c r="E24" s="9">
+        <f t="shared" si="0"/>
+        <v>-5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="11">
+        <f>F9/F6</f>
+        <v>0.121875</v>
+      </c>
+      <c r="D25" s="11">
+        <f>C25</f>
+        <v>0.121875</v>
+      </c>
+      <c r="E25" s="11">
+        <f>C25</f>
+        <v>0.121875</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="11">
+        <f>$F$11/$F$6</f>
+        <v>0.26874999999999999</v>
+      </c>
+      <c r="D26" s="11">
+        <f>$F$11/$F$6</f>
+        <v>0.26874999999999999</v>
+      </c>
+      <c r="E26" s="11">
+        <f>$F$11/$F$6</f>
+        <v>0.26874999999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="3">
+        <f t="shared" ref="C30:C41" si="1">INDEX($C15:$E15, MATCH($C$28, $C$14:$E$14, 0))</f>
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="str">
+        <f t="shared" ref="A31:A41" si="2">A16</f>
+        <v>Rev growth Y2</v>
+      </c>
+      <c r="C31" s="3">
+        <f t="shared" si="1"/>
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="str">
+        <f t="shared" si="2"/>
+        <v>Rev growth Y3</v>
+      </c>
+      <c r="C32" s="3">
+        <f t="shared" si="1"/>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="str">
+        <f t="shared" si="2"/>
+        <v>Rev growth Y4</v>
+      </c>
+      <c r="C33" s="3">
+        <f t="shared" si="1"/>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="str">
+        <f t="shared" si="2"/>
+        <v>Rev growth Y5</v>
+      </c>
+      <c r="C34" s="3">
+        <f t="shared" si="1"/>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="str">
+        <f t="shared" si="2"/>
+        <v>Operating Margin (Y1)</v>
+      </c>
+      <c r="C35" s="3">
+        <f t="shared" si="1"/>
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="str">
+        <f t="shared" si="2"/>
+        <v>Margin expansion / yr</v>
+      </c>
+      <c r="C36" s="3">
+        <f t="shared" si="1"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="str">
+        <f t="shared" si="2"/>
+        <v>Tax Rate</v>
+      </c>
+      <c r="C37" s="3">
+        <f t="shared" si="1"/>
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="str">
+        <f t="shared" si="2"/>
+        <v>Capex % of Revenue (Y1)</v>
+      </c>
+      <c r="C38" s="11">
+        <f t="shared" si="1"/>
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="str">
+        <f t="shared" si="2"/>
+        <v>Capex change / yr</v>
+      </c>
+      <c r="C39" s="11">
+        <f t="shared" si="1"/>
+        <v>-5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="str">
+        <f t="shared" si="2"/>
+        <v>D%A % of Revenue</v>
+      </c>
+      <c r="C40" s="11">
+        <f t="shared" si="1"/>
+        <v>0.121875</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="str">
+        <f t="shared" si="2"/>
+        <v>NWC % of Revenue</v>
+      </c>
+      <c r="C41" s="11">
+        <f t="shared" si="1"/>
+        <v>0.26874999999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44">
+        <v>2026</v>
+      </c>
+      <c r="D44">
+        <v>2027</v>
+      </c>
+      <c r="E44">
+        <v>2028</v>
+      </c>
+      <c r="F44">
+        <v>2029</v>
+      </c>
+      <c r="G44">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>5</v>
+      </c>
+      <c r="C45" s="7">
+        <f>F6*(1+C46)</f>
+        <v>3.3920000000000003</v>
+      </c>
+      <c r="D45" s="7">
+        <f>C45*(1+D46)</f>
+        <v>3.5955200000000005</v>
+      </c>
+      <c r="E45" s="7">
+        <f>D45*(1+E46)</f>
+        <v>3.7393408000000008</v>
+      </c>
+      <c r="F45" s="7">
+        <f>E45*(1+F46)</f>
+        <v>3.8889144320000009</v>
+      </c>
+      <c r="G45" s="7">
+        <f>F45*(1+G46)</f>
+        <v>4.0444710092800014</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>28</v>
+      </c>
+      <c r="C46" s="3">
+        <f>$C$30</f>
+        <v>0.06</v>
+      </c>
+      <c r="D46" s="3">
+        <f>$C$31</f>
+        <v>0.06</v>
+      </c>
+      <c r="E46" s="3">
+        <f>$C$32</f>
+        <v>0.04</v>
+      </c>
+      <c r="F46" s="3">
+        <f>$C$33</f>
+        <v>0.04</v>
+      </c>
+      <c r="G46" s="3">
+        <f>$C$34</f>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" s="11">
+        <f>$C$35</f>
+        <v>0.17</v>
+      </c>
+      <c r="D47" s="11">
+        <f>C47+$C$36</f>
+        <v>0.18000000000000002</v>
+      </c>
+      <c r="E47" s="11">
+        <f>D47+$C$36</f>
+        <v>0.19000000000000003</v>
+      </c>
+      <c r="F47" s="11">
+        <f>E47+$C$36</f>
+        <v>0.20000000000000004</v>
+      </c>
+      <c r="G47" s="11">
+        <f>F47+$C$36</f>
+        <v>0.21000000000000005</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>29</v>
+      </c>
+      <c r="C48" s="7">
+        <f>C45*C47</f>
+        <v>0.57664000000000015</v>
+      </c>
+      <c r="D48" s="7">
+        <f>D45*D47</f>
+        <v>0.64719360000000015</v>
+      </c>
+      <c r="E48" s="7">
+        <f>E45*E47</f>
+        <v>0.71047475200000021</v>
+      </c>
+      <c r="F48" s="7">
+        <f>F45*F47</f>
+        <v>0.77778288640000037</v>
+      </c>
+      <c r="G48" s="7">
+        <f>G45*G47</f>
+        <v>0.84933891194880051</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>30</v>
+      </c>
+      <c r="C49" s="7">
+        <f>C48*$C$37</f>
+        <v>8.0729600000000026E-2</v>
+      </c>
+      <c r="D49" s="7">
+        <f>D48*$C$37</f>
+        <v>9.0607104000000036E-2</v>
+      </c>
+      <c r="E49" s="7">
+        <f>E48*$C$37</f>
+        <v>9.9466465280000041E-2</v>
+      </c>
+      <c r="F49" s="7">
+        <f>F48*$C$37</f>
+        <v>0.10888960409600006</v>
+      </c>
+      <c r="G49" s="7">
+        <f>G48*$C$37</f>
+        <v>0.11890744767283208</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>31</v>
+      </c>
+      <c r="C50" s="7">
+        <f>C48-C49</f>
+        <v>0.49591040000000014</v>
+      </c>
+      <c r="D50" s="7">
+        <f>D48-D49</f>
+        <v>0.5565864960000001</v>
+      </c>
+      <c r="E50" s="7">
+        <f>E48-E49</f>
+        <v>0.61100828672000018</v>
+      </c>
+      <c r="F50" s="7">
+        <f>F48-F49</f>
+        <v>0.66889328230400036</v>
+      </c>
+      <c r="G50" s="7">
+        <f>G48-G49</f>
+        <v>0.73043146427596839</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>32</v>
+      </c>
+      <c r="C51" s="7">
+        <f>C45*$C$40</f>
+        <v>0.41340000000000005</v>
+      </c>
+      <c r="D51" s="7">
+        <f>D45*$C$40</f>
+        <v>0.43820400000000004</v>
+      </c>
+      <c r="E51" s="7">
+        <f>E45*$C$40</f>
+        <v>0.45573216000000011</v>
+      </c>
+      <c r="F51" s="7">
+        <f>F45*$C$40</f>
+        <v>0.4739614464000001</v>
+      </c>
+      <c r="G51" s="7">
+        <f>G45*$C$40</f>
+        <v>0.49291990425600013</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>22</v>
+      </c>
+      <c r="C52" s="11">
+        <f>$C$38</f>
+        <v>0.08</v>
+      </c>
+      <c r="D52" s="11">
+        <f>C52+$C$39</f>
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="E52" s="11">
+        <f>D52+$C$39</f>
+        <v>6.9999999999999993E-2</v>
+      </c>
+      <c r="F52" s="11">
+        <f>E52+$C$39</f>
+        <v>6.4999999999999988E-2</v>
+      </c>
+      <c r="G52" s="11">
+        <f>F52+$C$39</f>
+        <v>5.9999999999999991E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>33</v>
+      </c>
+      <c r="C53" s="7">
+        <f>C45*C52</f>
+        <v>0.27136000000000005</v>
+      </c>
+      <c r="D53" s="7">
+        <f>D45*D52</f>
+        <v>0.26966400000000001</v>
+      </c>
+      <c r="E53" s="7">
+        <f>E45*E52</f>
+        <v>0.26175385600000001</v>
+      </c>
+      <c r="F53" s="7">
+        <f>F45*F52</f>
+        <v>0.25277943808000003</v>
+      </c>
+      <c r="G53" s="7">
+        <f>G45*G52</f>
+        <v>0.24266826055680005</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>34</v>
+      </c>
+      <c r="C54" s="7">
+        <f>$C$41*(C45-F6)</f>
+        <v>5.1600000000000042E-2</v>
+      </c>
+      <c r="D54" s="7">
+        <f>$C$41*(D45-C45)</f>
+        <v>5.4696000000000036E-2</v>
+      </c>
+      <c r="E54" s="7">
+        <f>$C$41*(E45-D45)</f>
+        <v>3.8651840000000083E-2</v>
+      </c>
+      <c r="F54" s="7">
+        <f>$C$41*(F45-E45)</f>
+        <v>4.0197913600000017E-2</v>
+      </c>
+      <c r="G54" s="7">
+        <f>$C$41*(G45-F45)</f>
+        <v>4.1805830144000133E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>35</v>
+      </c>
+      <c r="C55" s="7">
+        <f>C50+C51-C53-C54</f>
+        <v>0.58635040000000005</v>
+      </c>
+      <c r="D55" s="7">
+        <f>D50+D51-D53-D54</f>
+        <v>0.67043049600000004</v>
+      </c>
+      <c r="E55" s="7">
+        <f>E50+E51-E53-E54</f>
+        <v>0.76633475072000024</v>
+      </c>
+      <c r="F55" s="7">
+        <f>F50+F51-F53-F54</f>
+        <v>0.84987737702400046</v>
+      </c>
+      <c r="G55" s="7">
+        <f>G50+G51-G53-G54</f>
+        <v>0.93887727783116848</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>37</v>
+      </c>
+      <c r="B58" s="3">
+        <f>0.0455</f>
+        <v>4.5499999999999999E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>38</v>
+      </c>
+      <c r="B59" s="3">
+        <f>0.05</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>39</v>
+      </c>
+      <c r="B60" s="10">
+        <v>1.31</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>40</v>
+      </c>
+      <c r="B61" s="3">
+        <f>B58+B59*B60</f>
+        <v>0.111</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>41</v>
+      </c>
+      <c r="B62" s="3">
+        <f>0.2/((4+3.72)/2)</f>
+        <v>5.181347150259067E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>21</v>
+      </c>
+      <c r="B63" s="3">
+        <f>C37</f>
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>42</v>
+      </c>
+      <c r="B64" s="3">
+        <f>B62*(1-B63)</f>
+        <v>4.4559585492227972E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>43</v>
+      </c>
+      <c r="B65">
+        <f>136.26*0.152</f>
+        <v>20.711519999999997</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>44</v>
+      </c>
+      <c r="B66">
+        <v>3.72</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>45</v>
+      </c>
+      <c r="B67">
+        <f>B65+B66</f>
+        <v>24.431519999999995</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>46</v>
+      </c>
+      <c r="B68" s="3">
+        <f>B65/B67</f>
+        <v>0.84773767657517829</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>47</v>
+      </c>
+      <c r="B69" s="3">
+        <f>B66/B67</f>
+        <v>0.15226232342482174</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>36</v>
+      </c>
+      <c r="B70" s="3">
+        <f>B68*B61+B69*B64</f>
+        <v>0.10088362811773841</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>48</v>
+      </c>
+      <c r="B71" s="9">
+        <v>2.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74">
+        <f>C44</f>
+        <v>2026</v>
+      </c>
+      <c r="D74">
+        <f>D44</f>
+        <v>2027</v>
+      </c>
+      <c r="E74">
+        <f>E44</f>
+        <v>2028</v>
+      </c>
+      <c r="F74">
+        <f>F44</f>
+        <v>2029</v>
+      </c>
+      <c r="G74">
+        <f>G44</f>
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>35</v>
+      </c>
+      <c r="C75" s="7">
+        <f>C55</f>
+        <v>0.58635040000000005</v>
+      </c>
+      <c r="D75" s="7">
+        <f>D55</f>
+        <v>0.67043049600000004</v>
+      </c>
+      <c r="E75" s="7">
+        <f>E55</f>
+        <v>0.76633475072000024</v>
+      </c>
+      <c r="F75" s="7">
+        <f>F55</f>
+        <v>0.84987737702400046</v>
+      </c>
+      <c r="G75" s="7">
+        <f>G55</f>
+        <v>0.93887727783116848</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>49</v>
+      </c>
+      <c r="C76">
+        <v>1</v>
+      </c>
+      <c r="D76">
+        <v>2</v>
+      </c>
+      <c r="E76">
+        <v>3</v>
+      </c>
+      <c r="F76">
+        <v>4</v>
+      </c>
+      <c r="G76">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>50</v>
+      </c>
+      <c r="C77" s="7">
+        <f>-PV($B$70, C76, 0, C75)</f>
+        <v>0.53261796708025033</v>
+      </c>
+      <c r="D77" s="7">
+        <f>-PV($B$70, D76, 0, D75)</f>
+        <v>0.55318568688709246</v>
+      </c>
+      <c r="E77" s="7">
+        <f>-PV($B$70, E76, 0, E75)</f>
+        <v>0.57437334906908399</v>
+      </c>
+      <c r="F77" s="7">
+        <f>-PV($B$70, F76, 0, F75)</f>
+        <v>0.57861623674112017</v>
+      </c>
+      <c r="G77" s="7">
+        <f>-PV($B$70, G76, 0, G75)</f>
+        <v>0.58063306403985737</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>51</v>
+      </c>
+      <c r="B79">
+        <f>(G75*(1+$B$71))/($B$70-$B$71)</f>
+        <v>12.681908254094017</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>52</v>
+      </c>
+      <c r="B80" s="10">
+        <f>-PV(B70, 5, 0, B79)</f>
+        <v>7.842915598572084</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>53</v>
+      </c>
+      <c r="B81" s="7">
+        <f>SUM(C77:G77)</f>
+        <v>2.8194263038174041</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>54</v>
+      </c>
+      <c r="B82" s="10">
+        <f>B80+B81</f>
+        <v>10.662341902389489</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>55</v>
+      </c>
+      <c r="B83">
+        <f>B80/B82</f>
+        <v>0.73557157239672122</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>54</v>
+      </c>
+      <c r="B85" s="10">
+        <f>B82</f>
+        <v>10.662341902389489</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>56</v>
+      </c>
+      <c r="B86">
+        <f>B66</f>
+        <v>3.72</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>57</v>
+      </c>
+      <c r="B87">
+        <f>360000000/1000000000</f>
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>43</v>
+      </c>
+      <c r="B88" s="10">
+        <f>B85-B86+B87</f>
+        <v>7.3023419023894887</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>58</v>
+      </c>
+      <c r="B89" s="10">
+        <f>152000000/1000000000</f>
+        <v>0.152</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>59</v>
+      </c>
+      <c r="B90">
+        <f>(B88)/B89</f>
+        <v>48.041723042036111</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>60</v>
+      </c>
+      <c r="B91">
+        <v>136.26</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>61</v>
+      </c>
+      <c r="B92">
+        <f>B90/B91-1</f>
+        <v>-0.64742607484194836</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>48</v>
+      </c>
+      <c r="C95" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="D95" s="9">
+        <v>2.2499999999999999E-2</v>
+      </c>
+      <c r="E95" s="9">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="F95" s="9">
+        <v>2.75E-2</v>
+      </c>
+      <c r="G95" s="3">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B96" s="11">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="C96" s="15">
+        <f t="shared" ref="C96:G102" si="3">(NPV($B96,$C$75:$G$75)+(($G$75*(1+C$95))/($B96-C$95))/(1+$B96)^5-$B$66+$B$87)/$B$89</f>
+        <v>61.74832863547325</v>
+      </c>
+      <c r="D96" s="15">
+        <f t="shared" si="3"/>
+        <v>64.491120942220078</v>
+      </c>
+      <c r="E96" s="15">
+        <f t="shared" si="3"/>
+        <v>67.462479274529159</v>
+      </c>
+      <c r="F96" s="15">
+        <f t="shared" si="3"/>
+        <v>70.692216592256415</v>
+      </c>
+      <c r="G96" s="15">
+        <f t="shared" si="3"/>
+        <v>74.215566393413425</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B97" s="11">
+        <f t="shared" ref="B97:B102" si="4">B96+0.5%</f>
+        <v>9.0000000000000011E-2</v>
+      </c>
+      <c r="C97" s="15">
+        <f t="shared" si="3"/>
+        <v>55.512012321922214</v>
+      </c>
+      <c r="D97" s="15">
+        <f t="shared" si="3"/>
+        <v>57.827259933004996</v>
+      </c>
+      <c r="E97" s="15">
+        <f t="shared" si="3"/>
+        <v>60.320603514171069</v>
+      </c>
+      <c r="F97" s="15">
+        <f t="shared" si="3"/>
+        <v>63.013414581830432</v>
+      </c>
+      <c r="G97" s="15">
+        <f t="shared" si="3"/>
+        <v>65.930626571794747</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B98" s="11">
+        <f t="shared" si="4"/>
+        <v>9.5000000000000015E-2</v>
+      </c>
+      <c r="C98" s="15">
+        <f t="shared" si="3"/>
+        <v>50.111268838501765</v>
+      </c>
+      <c r="D98" s="15">
+        <f t="shared" si="3"/>
+        <v>52.086643609207322</v>
+      </c>
+      <c r="E98" s="15">
+        <f t="shared" si="3"/>
+        <v>54.203116577820403</v>
+      </c>
+      <c r="F98" s="15">
+        <f t="shared" si="3"/>
+        <v>56.476365321886327</v>
+      </c>
+      <c r="G98" s="15">
+        <f t="shared" si="3"/>
+        <v>58.924479353957302</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B99" s="11">
+        <f t="shared" si="4"/>
+        <v>0.10000000000000002</v>
+      </c>
+      <c r="C99" s="15">
+        <f t="shared" si="3"/>
+        <v>45.389339500221084</v>
+      </c>
+      <c r="D99" s="15">
+        <f t="shared" si="3"/>
+        <v>47.090490321780969</v>
+      </c>
+      <c r="E99" s="15">
+        <f t="shared" si="3"/>
+        <v>48.905051198111522</v>
+      </c>
+      <c r="F99" s="15">
+        <f t="shared" si="3"/>
+        <v>50.844754203844197</v>
+      </c>
+      <c r="G99" s="15">
+        <f t="shared" si="3"/>
+        <v>52.923007424272036</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B100" s="11">
+        <f t="shared" si="4"/>
+        <v>0.10500000000000002</v>
+      </c>
+      <c r="C100" s="15">
+        <f t="shared" si="3"/>
+        <v>41.226352395187604</v>
+      </c>
+      <c r="D100" s="15">
+        <f t="shared" si="3"/>
+        <v>42.703361807964981</v>
+      </c>
+      <c r="E100" s="15">
+        <f t="shared" si="3"/>
+        <v>44.272684309040933</v>
+      </c>
+      <c r="F100" s="15">
+        <f t="shared" si="3"/>
+        <v>45.943253423089523</v>
+      </c>
+      <c r="G100" s="15">
+        <f t="shared" si="3"/>
+        <v>47.725193811408033</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B101" s="11">
+        <f t="shared" si="4"/>
+        <v>0.11000000000000003</v>
+      </c>
+      <c r="C101" s="15">
+        <f t="shared" si="3"/>
+        <v>37.529075984009246</v>
+      </c>
+      <c r="D101" s="15">
+        <f t="shared" si="3"/>
+        <v>38.820779291921383</v>
+      </c>
+      <c r="E101" s="15">
+        <f t="shared" si="3"/>
+        <v>40.188465147357768</v>
+      </c>
+      <c r="F101" s="15">
+        <f t="shared" si="3"/>
+        <v>41.639041054638774</v>
+      </c>
+      <c r="G101" s="15">
+        <f t="shared" si="3"/>
+        <v>43.180277956124847</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B102" s="11">
+        <f t="shared" si="4"/>
+        <v>0.11500000000000003</v>
+      </c>
+      <c r="C102" s="15">
+        <f t="shared" si="3"/>
+        <v>34.223908407337007</v>
+      </c>
+      <c r="D102" s="15">
+        <f t="shared" si="3"/>
+        <v>35.360855987849249</v>
+      </c>
+      <c r="E102" s="15">
+        <f t="shared" si="3"/>
+        <v>36.560967322834422</v>
+      </c>
+      <c r="F102" s="15">
+        <f t="shared" si="3"/>
+        <v>37.829656448390153</v>
+      </c>
+      <c r="G102" s="15">
+        <f t="shared" si="3"/>
+        <v>39.172974346037414</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>62</v>
+      </c>
+      <c r="B105" s="7">
+        <f>G48+G51</f>
+        <v>1.3422588162048006</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>63</v>
+      </c>
+      <c r="B106">
+        <f>B79/B105</f>
+        <v>9.4481839873115963</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>78</v>
+      </c>
+      <c r="B107">
+        <f>(B65+B66-B87)/(F7+F9)</f>
+        <v>28.319435294117639</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>65</v>
+      </c>
+      <c r="C110">
+        <v>8</v>
+      </c>
+      <c r="D110">
+        <v>12</v>
+      </c>
+      <c r="E110">
+        <v>16</v>
+      </c>
+      <c r="F110">
+        <v>20</v>
+      </c>
+      <c r="G110">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>66</v>
+      </c>
+      <c r="C111" s="14">
+        <f>(NPV($B$70,$C$75:$G$75)+(C110*$B$105)/(1+$B$70)^5-$B$66+$B$87)/$B$89</f>
+        <v>40.132945630042101</v>
+      </c>
+      <c r="D111" s="14">
+        <f>(NPV($B$70,$C$75:$G$75)+(D110*$B$105)/(1+$B$70)^5-$B$66+$B$87)/$B$89</f>
+        <v>61.977621393032209</v>
+      </c>
+      <c r="E111" s="14">
+        <f>(NPV($B$70,$C$75:$G$75)+(E110*$B$105)/(1+$B$70)^5-$B$66+$B$87)/$B$89</f>
+        <v>83.822297156022316</v>
+      </c>
+      <c r="F111" s="14">
+        <f>(NPV($B$70,$C$75:$G$75)+(F110*$B$105)/(1+$B$70)^5-$B$66+$B$87)/$B$89</f>
+        <v>105.66697291901247</v>
+      </c>
+      <c r="G111" s="14">
+        <f>(NPV($B$70,$C$75:$G$75)+(G110*$B$105)/(1+$B$70)^5-$B$66+$B$87)/$B$89</f>
+        <v>149.35632444499268</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>68</v>
+      </c>
+      <c r="B115" s="10">
+        <f>B91*B89</f>
+        <v>20.711519999999997</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>69</v>
+      </c>
+      <c r="B116" s="10">
+        <f>B115+B66-B87</f>
+        <v>24.071519999999996</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>70</v>
+      </c>
+      <c r="B117" s="10">
+        <f>(B116-B81)*(1+B70)^5</f>
+        <v>34.364401742569676</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>71</v>
+      </c>
+      <c r="B118" s="10">
+        <f>B117/B105</f>
+        <v>25.601919188531809</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>72</v>
+      </c>
+      <c r="B119" s="9">
+        <f>(B70*B117-G75*(1+0))/(B117+G75)</f>
+        <v>7.1606046752596797E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>